<commit_message>
BOM added some changes done in PCB mention in #5
</commit_message>
<xml_diff>
--- a/Design_Files/Deliverables/BOM/Client_BOM.xlsx
+++ b/Design_Files/Deliverables/BOM/Client_BOM.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="265">
   <si>
     <t>#</t>
   </si>
@@ -455,6 +455,9 @@
     <t>1K</t>
   </si>
   <si>
+    <t>R31 is DNP</t>
+  </si>
+  <si>
     <t>R2</t>
   </si>
   <si>
@@ -597,6 +600,9 @@
   </si>
   <si>
     <t>10K</t>
+  </si>
+  <si>
+    <t>R35 is DNP</t>
   </si>
   <si>
     <t>R17, R18</t>
@@ -819,7 +825,7 @@
     <numFmt numFmtId="179" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
     <numFmt numFmtId="180" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -900,6 +906,13 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1534,7 +1547,7 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1543,128 +1556,128 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1763,7 +1776,13 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="12" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="13" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1772,7 +1791,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="180" fontId="12" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="13" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3323,7 +3342,9 @@
         <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
-      <c r="R22" s="8"/>
+      <c r="R22" s="32" t="s">
+        <v>146</v>
+      </c>
       <c r="S22" s="31"/>
     </row>
     <row r="23" ht="36" spans="1:19">
@@ -3336,28 +3357,28 @@
         <v>139</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F23" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L23" s="11">
         <v>1</v>
@@ -3392,28 +3413,28 @@
         <v>139</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F24" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="L24" s="8">
         <v>1</v>
@@ -3448,28 +3469,28 @@
         <v>139</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L25" s="11">
         <v>2</v>
@@ -3504,28 +3525,28 @@
         <v>139</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F26" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L26" s="8">
         <v>1</v>
@@ -3560,28 +3581,28 @@
         <v>139</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F27" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L27" s="11">
         <v>1</v>
@@ -3616,16 +3637,16 @@
         <v>139</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>142</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H28" s="8" t="s">
         <v>54</v>
@@ -3634,10 +3655,10 @@
         <v>24</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L28" s="8">
         <v>2</v>
@@ -3672,28 +3693,28 @@
         <v>139</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F29" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K29" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L29" s="11">
         <v>1</v>
@@ -3728,28 +3749,28 @@
         <v>139</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>142</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L30" s="8">
         <v>2</v>
@@ -3784,28 +3805,28 @@
         <v>139</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F31" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K31" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L31" s="11">
         <v>10</v>
@@ -3827,7 +3848,9 @@
         <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
-      <c r="R31" s="11"/>
+      <c r="R31" s="33" t="s">
+        <v>195</v>
+      </c>
       <c r="S31" s="11"/>
     </row>
     <row r="32" ht="36" spans="1:19">
@@ -3840,28 +3863,28 @@
         <v>139</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>142</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="L32" s="8">
         <v>2</v>
@@ -3894,16 +3917,16 @@
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F33" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="H33" s="11" t="s">
         <v>54</v>
@@ -3912,10 +3935,10 @@
         <v>24</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="K33" s="11" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="L33" s="11">
         <v>3</v>
@@ -3950,16 +3973,16 @@
         <v>139</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>142</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H34" s="8" t="s">
         <v>54</v>
@@ -3968,10 +3991,10 @@
         <v>24</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="L34" s="8">
         <v>1</v>
@@ -4003,31 +4026,31 @@
         <v>33</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F35" s="11" t="s">
         <v>76</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J35" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="K35" s="11" t="s">
         <v>214</v>
-      </c>
-      <c r="K35" s="11" t="s">
-        <v>212</v>
       </c>
       <c r="L35" s="11">
         <v>1</v>
@@ -4059,31 +4082,31 @@
         <v>34</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J36" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="K36" s="8" t="s">
         <v>221</v>
-      </c>
-      <c r="K36" s="8" t="s">
-        <v>219</v>
       </c>
       <c r="L36" s="8">
         <v>1</v>
@@ -4115,31 +4138,31 @@
         <v>35</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J37" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="K37" s="11" t="s">
         <v>227</v>
-      </c>
-      <c r="K37" s="11" t="s">
-        <v>225</v>
       </c>
       <c r="L37" s="11">
         <v>1</v>
@@ -4171,31 +4194,31 @@
         <v>36</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J38" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="K38" s="8" t="s">
         <v>233</v>
-      </c>
-      <c r="K38" s="8" t="s">
-        <v>231</v>
       </c>
       <c r="L38" s="8">
         <v>1</v>
@@ -4228,28 +4251,28 @@
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="11" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J39" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="K39" s="11" t="s">
         <v>239</v>
-      </c>
-      <c r="K39" s="11" t="s">
-        <v>237</v>
       </c>
       <c r="L39" s="11">
         <v>1</v>
@@ -4281,31 +4304,31 @@
         <v>38</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J40" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="K40" s="8" t="s">
         <v>245</v>
-      </c>
-      <c r="K40" s="8" t="s">
-        <v>243</v>
       </c>
       <c r="L40" s="8">
         <v>1</v>
@@ -4337,31 +4360,31 @@
         <v>39</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="K41" s="11" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="L41" s="11">
         <v>1</v>
@@ -4393,31 +4416,31 @@
         <v>40</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J42" s="8" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="L42" s="8">
         <v>1</v>
@@ -4457,16 +4480,16 @@
       <c r="L43" s="17"/>
       <c r="M43" s="17"/>
       <c r="N43" s="28" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O43" s="29"/>
       <c r="P43" s="29"/>
-      <c r="Q43" s="32">
+      <c r="Q43" s="34">
         <f>SUM(Q3:Q42)</f>
         <v>29.0454</v>
       </c>
-      <c r="R43" s="33"/>
-      <c r="S43" s="34"/>
+      <c r="R43" s="35"/>
+      <c r="S43" s="36"/>
     </row>
     <row r="44" ht="19.5" spans="1:19">
       <c r="A44" s="2"/>
@@ -4483,16 +4506,16 @@
       <c r="L44" s="21"/>
       <c r="M44" s="21"/>
       <c r="N44" s="28" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="O44" s="29"/>
       <c r="P44" s="29"/>
-      <c r="Q44" s="35">
+      <c r="Q44" s="37">
         <f>Q43/1</f>
         <v>29.0454</v>
       </c>
-      <c r="R44" s="36"/>
-      <c r="S44" s="37"/>
+      <c r="R44" s="38"/>
+      <c r="S44" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>